<commit_message>
Fixed: #706 Split PreferencesView into 4 subviews (one per section)
</commit_message>
<xml_diff>
--- a/Photo Club Hub/Documentation/LineCount.xlsx
+++ b/Photo Club Hub/Documentation/LineCount.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/Photo Club Hub/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0294D82E-4EC0-754B-B495-B69E8712EC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A496D8EA-D987-0F42-A890-69C11ACB743E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
   </bookViews>
@@ -1305,6 +1305,9 @@
                 <c:pt idx="336">
                   <c:v>46096</c:v>
                 </c:pt>
+                <c:pt idx="337">
+                  <c:v>46097</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2324,6 +2327,9 @@
                 </c:pt>
                 <c:pt idx="336" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
                   <c:v>12919</c:v>
+                </c:pt>
+                <c:pt idx="337" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
+                  <c:v>13045</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3382,6 +3388,9 @@
                 <c:pt idx="336">
                   <c:v>46096</c:v>
                 </c:pt>
+                <c:pt idx="337">
+                  <c:v>46097</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4401,6 +4410,9 @@
                 </c:pt>
                 <c:pt idx="336">
                   <c:v>10348</c:v>
+                </c:pt>
+                <c:pt idx="337">
+                  <c:v>10433</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5461,6 +5473,9 @@
                 <c:pt idx="336">
                   <c:v>46096</c:v>
                 </c:pt>
+                <c:pt idx="337">
+                  <c:v>46097</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6480,6 +6495,9 @@
                 </c:pt>
                 <c:pt idx="336">
                   <c:v>1303</c:v>
+                </c:pt>
+                <c:pt idx="337">
+                  <c:v>1327</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7559,6 +7577,9 @@
                 <c:pt idx="336">
                   <c:v>46096</c:v>
                 </c:pt>
+                <c:pt idx="337">
+                  <c:v>46097</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -8578,6 +8599,9 @@
                 </c:pt>
                 <c:pt idx="336">
                   <c:v>1268</c:v>
+                </c:pt>
+                <c:pt idx="337">
+                  <c:v>1285</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10020,6 +10044,9 @@
                 <c:pt idx="336">
                   <c:v>46096</c:v>
                 </c:pt>
+                <c:pt idx="337">
+                  <c:v>46097</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -11038,7 +11065,10 @@
                   <c:v>119</c:v>
                 </c:pt>
                 <c:pt idx="336">
-                  <c:v>119</c:v>
+                  <c:v>121</c:v>
+                </c:pt>
+                <c:pt idx="337">
+                  <c:v>125</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12100,6 +12130,9 @@
                 <c:pt idx="336">
                   <c:v>46096</c:v>
                 </c:pt>
+                <c:pt idx="337">
+                  <c:v>46097</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -13118,6 +13151,9 @@
                   <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="336">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="337">
                   <c:v>31</c:v>
                 </c:pt>
               </c:numCache>
@@ -14946,7 +14982,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B9E993F-B784-7448-B38E-9BEFCF4E7032}">
-  <dimension ref="A1:Q339"/>
+  <dimension ref="A1:Q340"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -29181,7 +29217,7 @@
         <v>197</v>
       </c>
       <c r="G339" s="4">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H339" s="16">
         <f t="shared" ref="H339" si="516">SUM(I339:K339)</f>
@@ -29200,6 +29236,49 @@
       <c r="M339" s="19"/>
       <c r="N339" s="19"/>
       <c r="O339">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="340" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A340" s="1">
+        <v>46097</v>
+      </c>
+      <c r="B340" s="2">
+        <v>9</v>
+      </c>
+      <c r="C340">
+        <f t="shared" ref="C340" si="517">SUM(D340:F340)</f>
+        <v>1673</v>
+      </c>
+      <c r="D340">
+        <v>1105</v>
+      </c>
+      <c r="E340">
+        <v>371</v>
+      </c>
+      <c r="F340" s="3">
+        <v>197</v>
+      </c>
+      <c r="G340" s="4">
+        <v>125</v>
+      </c>
+      <c r="H340" s="16">
+        <f t="shared" ref="H340" si="518">SUM(I340:K340)</f>
+        <v>13045</v>
+      </c>
+      <c r="I340" s="5">
+        <v>10433</v>
+      </c>
+      <c r="J340" s="6">
+        <v>1327</v>
+      </c>
+      <c r="K340" s="7">
+        <v>1285</v>
+      </c>
+      <c r="L340" s="19"/>
+      <c r="M340" s="19"/>
+      <c r="N340" s="19"/>
+      <c r="O340">
         <v>31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chooseImageURL is now a separate file
</commit_message>
<xml_diff>
--- a/Photo Club Hub/Documentation/LineCount.xlsx
+++ b/Photo Club Hub/Documentation/LineCount.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/Photo Club Hub/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA219F1C-E8AE-0B48-B63C-46952C73B74F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C18A1DA-1064-0941-B457-BAFF03C48EFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="25620" windowHeight="26400" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="1" r:id="rId1"/>
@@ -1311,6 +1311,9 @@
                 <c:pt idx="338">
                   <c:v>46100</c:v>
                 </c:pt>
+                <c:pt idx="339">
+                  <c:v>46103</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2336,6 +2339,9 @@
                 </c:pt>
                 <c:pt idx="338" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
                   <c:v>13146</c:v>
+                </c:pt>
+                <c:pt idx="339" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
+                  <c:v>13142</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3400,6 +3406,9 @@
                 <c:pt idx="338">
                   <c:v>46100</c:v>
                 </c:pt>
+                <c:pt idx="339">
+                  <c:v>46103</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4425,6 +4434,9 @@
                 </c:pt>
                 <c:pt idx="338">
                   <c:v>10523</c:v>
+                </c:pt>
+                <c:pt idx="339">
+                  <c:v>10511</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5491,6 +5503,9 @@
                 <c:pt idx="338">
                   <c:v>46100</c:v>
                 </c:pt>
+                <c:pt idx="339">
+                  <c:v>46103</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6516,6 +6531,9 @@
                 </c:pt>
                 <c:pt idx="338">
                   <c:v>1326</c:v>
+                </c:pt>
+                <c:pt idx="339">
+                  <c:v>1331</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7601,6 +7619,9 @@
                 <c:pt idx="338">
                   <c:v>46100</c:v>
                 </c:pt>
+                <c:pt idx="339">
+                  <c:v>46103</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -8626,6 +8647,9 @@
                 </c:pt>
                 <c:pt idx="338">
                   <c:v>1297</c:v>
+                </c:pt>
+                <c:pt idx="339">
+                  <c:v>1300</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10074,6 +10098,9 @@
                 <c:pt idx="338">
                   <c:v>46100</c:v>
                 </c:pt>
+                <c:pt idx="339">
+                  <c:v>46103</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -11099,6 +11126,9 @@
                 </c:pt>
                 <c:pt idx="338">
                   <c:v>125</c:v>
+                </c:pt>
+                <c:pt idx="339">
+                  <c:v>126</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12166,6 +12196,9 @@
                 <c:pt idx="338">
                   <c:v>46100</c:v>
                 </c:pt>
+                <c:pt idx="339">
+                  <c:v>46103</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -13190,6 +13223,9 @@
                   <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="338">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="339">
                   <c:v>31</c:v>
                 </c:pt>
               </c:numCache>
@@ -15018,7 +15054,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B9E993F-B784-7448-B38E-9BEFCF4E7032}">
-  <dimension ref="A1:Q341"/>
+  <dimension ref="A1:Q342"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -29358,6 +29394,49 @@
       <c r="M341" s="19"/>
       <c r="N341" s="19"/>
       <c r="O341">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="342" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A342" s="1">
+        <v>46103</v>
+      </c>
+      <c r="B342" s="2">
+        <v>9</v>
+      </c>
+      <c r="C342">
+        <f t="shared" ref="C342" si="521">SUM(D342:F342)</f>
+        <v>1673</v>
+      </c>
+      <c r="D342">
+        <v>1105</v>
+      </c>
+      <c r="E342">
+        <v>371</v>
+      </c>
+      <c r="F342" s="3">
+        <v>197</v>
+      </c>
+      <c r="G342" s="4">
+        <v>126</v>
+      </c>
+      <c r="H342" s="16">
+        <f t="shared" ref="H342" si="522">SUM(I342:K342)</f>
+        <v>13142</v>
+      </c>
+      <c r="I342" s="5">
+        <v>10511</v>
+      </c>
+      <c r="J342" s="6">
+        <v>1331</v>
+      </c>
+      <c r="K342" s="7">
+        <v>1300</v>
+      </c>
+      <c r="L342" s="19"/>
+      <c r="M342" s="19"/>
+      <c r="N342" s="19"/>
+      <c r="O342">
         <v>31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Merged SectionHeader1718 and SectionHeader2626 into SectionHeader
</commit_message>
<xml_diff>
--- a/Photo Club Hub/Documentation/LineCount.xlsx
+++ b/Photo Club Hub/Documentation/LineCount.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/Photo Club Hub/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B40B176A-38CA-644B-A8E7-7653A4935245}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D5E9492-BEC6-EC4A-AF0E-59BAD07F699E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="25620" windowHeight="26400" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="25620" windowHeight="26400" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="1" r:id="rId1"/>
@@ -1317,6 +1317,9 @@
                 <c:pt idx="340">
                   <c:v>46105</c:v>
                 </c:pt>
+                <c:pt idx="341">
+                  <c:v>46106</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2348,6 +2351,9 @@
                 </c:pt>
                 <c:pt idx="340" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
                   <c:v>13437</c:v>
+                </c:pt>
+                <c:pt idx="341" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
+                  <c:v>13680</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3418,6 +3424,9 @@
                 <c:pt idx="340">
                   <c:v>46105</c:v>
                 </c:pt>
+                <c:pt idx="341">
+                  <c:v>46106</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4449,6 +4458,9 @@
                 </c:pt>
                 <c:pt idx="340">
                   <c:v>10757</c:v>
+                </c:pt>
+                <c:pt idx="341">
+                  <c:v>10954</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5521,6 +5533,9 @@
                 <c:pt idx="340">
                   <c:v>46105</c:v>
                 </c:pt>
+                <c:pt idx="341">
+                  <c:v>46106</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6552,6 +6567,9 @@
                 </c:pt>
                 <c:pt idx="340">
                   <c:v>1360</c:v>
+                </c:pt>
+                <c:pt idx="341">
+                  <c:v>1387</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7643,6 +7661,9 @@
                 <c:pt idx="340">
                   <c:v>46105</c:v>
                 </c:pt>
+                <c:pt idx="341">
+                  <c:v>46106</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -8674,6 +8695,9 @@
                 </c:pt>
                 <c:pt idx="340">
                   <c:v>1320</c:v>
+                </c:pt>
+                <c:pt idx="341">
+                  <c:v>1339</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10128,6 +10152,9 @@
                 <c:pt idx="340">
                   <c:v>46105</c:v>
                 </c:pt>
+                <c:pt idx="341">
+                  <c:v>46106</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -11158,6 +11185,9 @@
                   <c:v>126</c:v>
                 </c:pt>
                 <c:pt idx="340">
+                  <c:v>131</c:v>
+                </c:pt>
+                <c:pt idx="341">
                   <c:v>131</c:v>
                 </c:pt>
               </c:numCache>
@@ -12232,6 +12262,9 @@
                 <c:pt idx="340">
                   <c:v>46105</c:v>
                 </c:pt>
+                <c:pt idx="341">
+                  <c:v>46106</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -13262,6 +13295,9 @@
                   <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="340">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="341">
                   <c:v>31</c:v>
                 </c:pt>
               </c:numCache>
@@ -15090,7 +15126,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B9E993F-B784-7448-B38E-9BEFCF4E7032}">
-  <dimension ref="A1:Q343"/>
+  <dimension ref="A1:Q344"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -29516,6 +29552,49 @@
       <c r="M343" s="19"/>
       <c r="N343" s="19"/>
       <c r="O343">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="344" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A344" s="1">
+        <v>46106</v>
+      </c>
+      <c r="B344" s="2">
+        <v>9</v>
+      </c>
+      <c r="C344">
+        <f t="shared" ref="C344" si="525">SUM(D344:F344)</f>
+        <v>1673</v>
+      </c>
+      <c r="D344">
+        <v>1105</v>
+      </c>
+      <c r="E344">
+        <v>371</v>
+      </c>
+      <c r="F344" s="3">
+        <v>197</v>
+      </c>
+      <c r="G344" s="4">
+        <v>131</v>
+      </c>
+      <c r="H344" s="16">
+        <f t="shared" ref="H344" si="526">SUM(I344:K344)</f>
+        <v>13680</v>
+      </c>
+      <c r="I344" s="5">
+        <v>10954</v>
+      </c>
+      <c r="J344" s="6">
+        <v>1387</v>
+      </c>
+      <c r="K344" s="7">
+        <v>1339</v>
+      </c>
+      <c r="L344" s="19"/>
+      <c r="M344" s="19"/>
+      <c r="N344" s="19"/>
+      <c r="O344">
         <v>31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Merged ReadmeSection1718 and ReadmeSection2626
</commit_message>
<xml_diff>
--- a/Photo Club Hub/Documentation/LineCount.xlsx
+++ b/Photo Club Hub/Documentation/LineCount.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/Photo Club Hub/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D5E9492-BEC6-EC4A-AF0E-59BAD07F699E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9FD515E-DEFD-EC40-9F0A-FCC748777649}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="25620" windowHeight="26400" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="1" r:id="rId1"/>
@@ -2353,7 +2353,7 @@
                   <c:v>13437</c:v>
                 </c:pt>
                 <c:pt idx="341" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
-                  <c:v>13680</c:v>
+                  <c:v>13642</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4460,7 +4460,7 @@
                   <c:v>10757</c:v>
                 </c:pt>
                 <c:pt idx="341">
-                  <c:v>10954</c:v>
+                  <c:v>10928</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6569,7 +6569,7 @@
                   <c:v>1360</c:v>
                 </c:pt>
                 <c:pt idx="341">
-                  <c:v>1387</c:v>
+                  <c:v>1377</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8697,7 +8697,7 @@
                   <c:v>1320</c:v>
                 </c:pt>
                 <c:pt idx="341">
-                  <c:v>1339</c:v>
+                  <c:v>1337</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -29580,16 +29580,16 @@
       </c>
       <c r="H344" s="16">
         <f t="shared" ref="H344" si="526">SUM(I344:K344)</f>
-        <v>13680</v>
+        <v>13642</v>
       </c>
       <c r="I344" s="5">
-        <v>10954</v>
+        <v>10928</v>
       </c>
       <c r="J344" s="6">
-        <v>1387</v>
+        <v>1377</v>
       </c>
       <c r="K344" s="7">
-        <v>1339</v>
+        <v>1337</v>
       </c>
       <c r="L344" s="19"/>
       <c r="M344" s="19"/>

</xml_diff>

<commit_message>
Factored out ReadmeCaptionedImage file
</commit_message>
<xml_diff>
--- a/Photo Club Hub/Documentation/LineCount.xlsx
+++ b/Photo Club Hub/Documentation/LineCount.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/Photo Club Hub/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9FD515E-DEFD-EC40-9F0A-FCC748777649}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5D77EA3-1A39-684A-BF30-486F14206E4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="25620" windowHeight="26400" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="1" r:id="rId1"/>
@@ -2353,7 +2353,7 @@
                   <c:v>13437</c:v>
                 </c:pt>
                 <c:pt idx="341" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
-                  <c:v>13642</c:v>
+                  <c:v>13518</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4460,7 +4460,7 @@
                   <c:v>10757</c:v>
                 </c:pt>
                 <c:pt idx="341">
-                  <c:v>10928</c:v>
+                  <c:v>10812</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6569,7 +6569,7 @@
                   <c:v>1360</c:v>
                 </c:pt>
                 <c:pt idx="341">
-                  <c:v>1377</c:v>
+                  <c:v>1371</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8697,7 +8697,7 @@
                   <c:v>1320</c:v>
                 </c:pt>
                 <c:pt idx="341">
-                  <c:v>1337</c:v>
+                  <c:v>1335</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11188,7 +11188,7 @@
                   <c:v>131</c:v>
                 </c:pt>
                 <c:pt idx="341">
-                  <c:v>131</c:v>
+                  <c:v>133</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -29576,20 +29576,20 @@
         <v>197</v>
       </c>
       <c r="G344" s="4">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H344" s="16">
         <f t="shared" ref="H344" si="526">SUM(I344:K344)</f>
-        <v>13642</v>
+        <v>13518</v>
       </c>
       <c r="I344" s="5">
-        <v>10928</v>
+        <v>10812</v>
       </c>
       <c r="J344" s="6">
-        <v>1377</v>
+        <v>1371</v>
       </c>
       <c r="K344" s="7">
-        <v>1337</v>
+        <v>1335</v>
       </c>
       <c r="L344" s="19"/>
       <c r="M344" s="19"/>

</xml_diff>

<commit_message>
Merge ReadmeSectionOnSupportedPlatforms1718 and ReadmeSectionOnSupportedPlatforms2626
</commit_message>
<xml_diff>
--- a/Photo Club Hub/Documentation/LineCount.xlsx
+++ b/Photo Club Hub/Documentation/LineCount.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/Photo Club Hub/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5D77EA3-1A39-684A-BF30-486F14206E4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09FB7FC2-5C64-054F-BA1A-41C95EAD9493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="25620" windowHeight="26400" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
   </bookViews>
@@ -1320,6 +1320,9 @@
                 <c:pt idx="341">
                   <c:v>46106</c:v>
                 </c:pt>
+                <c:pt idx="342">
+                  <c:v>46107</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2354,6 +2357,9 @@
                 </c:pt>
                 <c:pt idx="341" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
                   <c:v>13518</c:v>
+                </c:pt>
+                <c:pt idx="342" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
+                  <c:v>13116</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3427,6 +3433,9 @@
                 <c:pt idx="341">
                   <c:v>46106</c:v>
                 </c:pt>
+                <c:pt idx="342">
+                  <c:v>46107</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4461,6 +4470,9 @@
                 </c:pt>
                 <c:pt idx="341">
                   <c:v>10812</c:v>
+                </c:pt>
+                <c:pt idx="342">
+                  <c:v>10422</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5536,6 +5548,9 @@
                 <c:pt idx="341">
                   <c:v>46106</c:v>
                 </c:pt>
+                <c:pt idx="342">
+                  <c:v>46107</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6570,6 +6585,9 @@
                 </c:pt>
                 <c:pt idx="341">
                   <c:v>1371</c:v>
+                </c:pt>
+                <c:pt idx="342">
+                  <c:v>1358</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7664,6 +7682,9 @@
                 <c:pt idx="341">
                   <c:v>46106</c:v>
                 </c:pt>
+                <c:pt idx="342">
+                  <c:v>46107</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -8698,6 +8719,9 @@
                 </c:pt>
                 <c:pt idx="341">
                   <c:v>1335</c:v>
+                </c:pt>
+                <c:pt idx="342">
+                  <c:v>1336</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10155,6 +10179,9 @@
                 <c:pt idx="341">
                   <c:v>46106</c:v>
                 </c:pt>
+                <c:pt idx="342">
+                  <c:v>46107</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -11189,6 +11216,9 @@
                 </c:pt>
                 <c:pt idx="341">
                   <c:v>133</c:v>
+                </c:pt>
+                <c:pt idx="342">
+                  <c:v>131</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12265,6 +12295,9 @@
                 <c:pt idx="341">
                   <c:v>46106</c:v>
                 </c:pt>
+                <c:pt idx="342">
+                  <c:v>46107</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -13298,6 +13331,9 @@
                   <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="341">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="342">
                   <c:v>31</c:v>
                 </c:pt>
               </c:numCache>
@@ -15126,7 +15162,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B9E993F-B784-7448-B38E-9BEFCF4E7032}">
-  <dimension ref="A1:Q344"/>
+  <dimension ref="A1:Q345"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -29595,6 +29631,49 @@
       <c r="M344" s="19"/>
       <c r="N344" s="19"/>
       <c r="O344">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="345" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A345" s="1">
+        <v>46107</v>
+      </c>
+      <c r="B345" s="2">
+        <v>9</v>
+      </c>
+      <c r="C345">
+        <f t="shared" ref="C345" si="527">SUM(D345:F345)</f>
+        <v>1673</v>
+      </c>
+      <c r="D345">
+        <v>1105</v>
+      </c>
+      <c r="E345">
+        <v>371</v>
+      </c>
+      <c r="F345" s="3">
+        <v>197</v>
+      </c>
+      <c r="G345" s="4">
+        <v>131</v>
+      </c>
+      <c r="H345" s="16">
+        <f t="shared" ref="H345" si="528">SUM(I345:K345)</f>
+        <v>13116</v>
+      </c>
+      <c r="I345" s="5">
+        <v>10422</v>
+      </c>
+      <c r="J345" s="6">
+        <v>1358</v>
+      </c>
+      <c r="K345" s="7">
+        <v>1336</v>
+      </c>
+      <c r="L345" s="19"/>
+      <c r="M345" s="19"/>
+      <c r="N345" s="19"/>
+      <c r="O345">
         <v>31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Merged ReadmeView1718 and ReadmeView2626 Fixed: #713
</commit_message>
<xml_diff>
--- a/Photo Club Hub/Documentation/LineCount.xlsx
+++ b/Photo Club Hub/Documentation/LineCount.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/Photo Club Hub/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09FB7FC2-5C64-054F-BA1A-41C95EAD9493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA577389-A979-1B4F-80FC-A0F86F662163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="25620" windowHeight="26400" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="1" r:id="rId1"/>
@@ -2359,7 +2359,7 @@
                   <c:v>13518</c:v>
                 </c:pt>
                 <c:pt idx="342" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
-                  <c:v>13116</c:v>
+                  <c:v>12940</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4472,7 +4472,7 @@
                   <c:v>10812</c:v>
                 </c:pt>
                 <c:pt idx="342">
-                  <c:v>10422</c:v>
+                  <c:v>10263</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6587,7 +6587,7 @@
                   <c:v>1371</c:v>
                 </c:pt>
                 <c:pt idx="342">
-                  <c:v>1358</c:v>
+                  <c:v>1345</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8721,7 +8721,7 @@
                   <c:v>1335</c:v>
                 </c:pt>
                 <c:pt idx="342">
-                  <c:v>1336</c:v>
+                  <c:v>1332</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11218,7 +11218,7 @@
                   <c:v>133</c:v>
                 </c:pt>
                 <c:pt idx="342">
-                  <c:v>131</c:v>
+                  <c:v>129</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -29655,20 +29655,20 @@
         <v>197</v>
       </c>
       <c r="G345" s="4">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H345" s="16">
         <f t="shared" ref="H345" si="528">SUM(I345:K345)</f>
-        <v>13116</v>
+        <v>12940</v>
       </c>
       <c r="I345" s="5">
-        <v>10422</v>
+        <v>10263</v>
       </c>
       <c r="J345" s="6">
-        <v>1358</v>
+        <v>1345</v>
       </c>
       <c r="K345" s="7">
-        <v>1336</v>
+        <v>1332</v>
       </c>
       <c r="L345" s="19"/>
       <c r="M345" s="19"/>

</xml_diff>

<commit_message>
Fix: #702 But works for Member screen only
</commit_message>
<xml_diff>
--- a/Photo Club Hub/Documentation/LineCount.xlsx
+++ b/Photo Club Hub/Documentation/LineCount.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/Photo Club Hub/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F141935E-E7C2-1F43-8046-3E2DA72AB2E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1607982-CEA5-9540-81B5-F9D231BD44F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="33800" windowHeight="26400" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="1" r:id="rId1"/>
@@ -1326,6 +1326,9 @@
                 <c:pt idx="343">
                   <c:v>46110</c:v>
                 </c:pt>
+                <c:pt idx="344">
+                  <c:v>46113</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2366,6 +2369,9 @@
                 </c:pt>
                 <c:pt idx="343" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
                   <c:v>13093</c:v>
+                </c:pt>
+                <c:pt idx="344" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
+                  <c:v>13157</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3445,6 +3451,9 @@
                 <c:pt idx="343">
                   <c:v>46110</c:v>
                 </c:pt>
+                <c:pt idx="344">
+                  <c:v>46113</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4485,6 +4494,9 @@
                 </c:pt>
                 <c:pt idx="343">
                   <c:v>10381</c:v>
+                </c:pt>
+                <c:pt idx="344">
+                  <c:v>10411</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5566,6 +5578,9 @@
                 <c:pt idx="343">
                   <c:v>46110</c:v>
                 </c:pt>
+                <c:pt idx="344">
+                  <c:v>46113</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6606,6 +6621,9 @@
                 </c:pt>
                 <c:pt idx="343">
                   <c:v>1368</c:v>
+                </c:pt>
+                <c:pt idx="344">
+                  <c:v>1403</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7706,6 +7724,9 @@
                 <c:pt idx="343">
                   <c:v>46110</c:v>
                 </c:pt>
+                <c:pt idx="344">
+                  <c:v>46113</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -8746,6 +8767,9 @@
                 </c:pt>
                 <c:pt idx="343">
                   <c:v>1344</c:v>
+                </c:pt>
+                <c:pt idx="344">
+                  <c:v>1343</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10209,6 +10233,9 @@
                 <c:pt idx="343">
                   <c:v>46110</c:v>
                 </c:pt>
+                <c:pt idx="344">
+                  <c:v>46113</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -11248,6 +11275,9 @@
                   <c:v>129</c:v>
                 </c:pt>
                 <c:pt idx="343">
+                  <c:v>129</c:v>
+                </c:pt>
+                <c:pt idx="344">
                   <c:v>129</c:v>
                 </c:pt>
               </c:numCache>
@@ -12331,6 +12361,9 @@
                 <c:pt idx="343">
                   <c:v>46110</c:v>
                 </c:pt>
+                <c:pt idx="344">
+                  <c:v>46113</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -13370,6 +13403,9 @@
                   <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="343">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="344">
                   <c:v>31</c:v>
                 </c:pt>
               </c:numCache>
@@ -15198,7 +15234,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B9E993F-B784-7448-B38E-9BEFCF4E7032}">
-  <dimension ref="A1:Q346"/>
+  <dimension ref="A1:Q347"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -29753,6 +29789,49 @@
       <c r="M346" s="19"/>
       <c r="N346" s="19"/>
       <c r="O346">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="347" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A347" s="1">
+        <v>46113</v>
+      </c>
+      <c r="B347" s="2">
+        <v>9</v>
+      </c>
+      <c r="C347">
+        <f t="shared" ref="C347" si="531">SUM(D347:F347)</f>
+        <v>1673</v>
+      </c>
+      <c r="D347">
+        <v>1105</v>
+      </c>
+      <c r="E347">
+        <v>371</v>
+      </c>
+      <c r="F347" s="3">
+        <v>197</v>
+      </c>
+      <c r="G347" s="4">
+        <v>129</v>
+      </c>
+      <c r="H347" s="16">
+        <f t="shared" ref="H347" si="532">SUM(I347:K347)</f>
+        <v>13157</v>
+      </c>
+      <c r="I347" s="5">
+        <v>10411</v>
+      </c>
+      <c r="J347" s="6">
+        <v>1403</v>
+      </c>
+      <c r="K347" s="7">
+        <v>1343</v>
+      </c>
+      <c r="L347" s="19"/>
+      <c r="M347" s="19"/>
+      <c r="N347" s="19"/>
+      <c r="O347">
         <v>31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: #720 Restructured layout and tappable links in MemberPortfolioRow view.
</commit_message>
<xml_diff>
--- a/Photo Club Hub/Documentation/LineCount.xlsx
+++ b/Photo Club Hub/Documentation/LineCount.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/Photo Club Hub/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1607982-CEA5-9540-81B5-F9D231BD44F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09571784-1749-E248-BBA3-3023EB5B701E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="33800" windowHeight="26400" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
   </bookViews>
@@ -1329,6 +1329,9 @@
                 <c:pt idx="344">
                   <c:v>46113</c:v>
                 </c:pt>
+                <c:pt idx="345">
+                  <c:v>46114</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2372,6 +2375,9 @@
                 </c:pt>
                 <c:pt idx="344" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
                   <c:v>13157</c:v>
+                </c:pt>
+                <c:pt idx="345" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
+                  <c:v>13206</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3454,6 +3460,9 @@
                 <c:pt idx="344">
                   <c:v>46113</c:v>
                 </c:pt>
+                <c:pt idx="345">
+                  <c:v>46114</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4497,6 +4506,9 @@
                 </c:pt>
                 <c:pt idx="344">
                   <c:v>10411</c:v>
+                </c:pt>
+                <c:pt idx="345">
+                  <c:v>10428</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5581,6 +5593,9 @@
                 <c:pt idx="344">
                   <c:v>46113</c:v>
                 </c:pt>
+                <c:pt idx="345">
+                  <c:v>46114</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6624,6 +6639,9 @@
                 </c:pt>
                 <c:pt idx="344">
                   <c:v>1403</c:v>
+                </c:pt>
+                <c:pt idx="345">
+                  <c:v>1423</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7727,6 +7745,9 @@
                 <c:pt idx="344">
                   <c:v>46113</c:v>
                 </c:pt>
+                <c:pt idx="345">
+                  <c:v>46114</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -8770,6 +8791,9 @@
                 </c:pt>
                 <c:pt idx="344">
                   <c:v>1343</c:v>
+                </c:pt>
+                <c:pt idx="345">
+                  <c:v>1355</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10236,6 +10260,9 @@
                 <c:pt idx="344">
                   <c:v>46113</c:v>
                 </c:pt>
+                <c:pt idx="345">
+                  <c:v>46114</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -11279,6 +11306,9 @@
                 </c:pt>
                 <c:pt idx="344">
                   <c:v>129</c:v>
+                </c:pt>
+                <c:pt idx="345">
+                  <c:v>130</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12364,6 +12394,9 @@
                 <c:pt idx="344">
                   <c:v>46113</c:v>
                 </c:pt>
+                <c:pt idx="345">
+                  <c:v>46114</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -13406,6 +13439,9 @@
                   <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="344">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="345">
                   <c:v>31</c:v>
                 </c:pt>
               </c:numCache>
@@ -15234,7 +15270,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B9E993F-B784-7448-B38E-9BEFCF4E7032}">
-  <dimension ref="A1:Q347"/>
+  <dimension ref="A1:Q348"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -29832,6 +29868,49 @@
       <c r="M347" s="19"/>
       <c r="N347" s="19"/>
       <c r="O347">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="348" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A348" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B348" s="2">
+        <v>9</v>
+      </c>
+      <c r="C348">
+        <f t="shared" ref="C348" si="533">SUM(D348:F348)</f>
+        <v>1673</v>
+      </c>
+      <c r="D348">
+        <v>1105</v>
+      </c>
+      <c r="E348">
+        <v>371</v>
+      </c>
+      <c r="F348" s="3">
+        <v>197</v>
+      </c>
+      <c r="G348" s="4">
+        <v>130</v>
+      </c>
+      <c r="H348" s="16">
+        <f t="shared" ref="H348" si="534">SUM(I348:K348)</f>
+        <v>13206</v>
+      </c>
+      <c r="I348" s="5">
+        <v>10428</v>
+      </c>
+      <c r="J348" s="6">
+        <v>1423</v>
+      </c>
+      <c r="K348" s="7">
+        <v>1355</v>
+      </c>
+      <c r="L348" s="19"/>
+      <c r="M348" s="19"/>
+      <c r="N348" s="19"/>
+      <c r="O348">
         <v>31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Minor: renamed a parameter membership > member
</commit_message>
<xml_diff>
--- a/Photo Club Hub/Documentation/LineCount.xlsx
+++ b/Photo Club Hub/Documentation/LineCount.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/Photo Club Hub/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4E01D72-6371-C441-9854-1D71EC8BDCC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6A926F7-D56A-1144-954D-7E0749593B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="33800" windowHeight="26400" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
   </bookViews>
@@ -1338,6 +1338,9 @@
                 <c:pt idx="347">
                   <c:v>46118</c:v>
                 </c:pt>
+                <c:pt idx="348">
+                  <c:v>46120</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2390,6 +2393,9 @@
                 </c:pt>
                 <c:pt idx="347" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
                   <c:v>13002</c:v>
+                </c:pt>
+                <c:pt idx="348" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
+                  <c:v>13429</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3481,6 +3487,9 @@
                 <c:pt idx="347">
                   <c:v>46118</c:v>
                 </c:pt>
+                <c:pt idx="348">
+                  <c:v>46120</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4533,6 +4542,9 @@
                 </c:pt>
                 <c:pt idx="347">
                   <c:v>10105</c:v>
+                </c:pt>
+                <c:pt idx="348">
+                  <c:v>10445</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5626,6 +5638,9 @@
                 <c:pt idx="347">
                   <c:v>46118</c:v>
                 </c:pt>
+                <c:pt idx="348">
+                  <c:v>46120</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6678,6 +6693,9 @@
                 </c:pt>
                 <c:pt idx="347">
                   <c:v>1499</c:v>
+                </c:pt>
+                <c:pt idx="348">
+                  <c:v>1539</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7790,6 +7808,9 @@
                 <c:pt idx="347">
                   <c:v>46118</c:v>
                 </c:pt>
+                <c:pt idx="348">
+                  <c:v>46120</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -8842,6 +8863,9 @@
                 </c:pt>
                 <c:pt idx="347">
                   <c:v>1398</c:v>
+                </c:pt>
+                <c:pt idx="348">
+                  <c:v>1445</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10317,6 +10341,9 @@
                 <c:pt idx="347">
                   <c:v>46118</c:v>
                 </c:pt>
+                <c:pt idx="348">
+                  <c:v>46120</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -11368,6 +11395,9 @@
                   <c:v>132</c:v>
                 </c:pt>
                 <c:pt idx="347">
+                  <c:v>132</c:v>
+                </c:pt>
+                <c:pt idx="348">
                   <c:v>132</c:v>
                 </c:pt>
               </c:numCache>
@@ -12463,6 +12493,9 @@
                 <c:pt idx="347">
                   <c:v>46118</c:v>
                 </c:pt>
+                <c:pt idx="348">
+                  <c:v>46120</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -13514,6 +13547,9 @@
                   <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="347">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="348">
                   <c:v>31</c:v>
                 </c:pt>
               </c:numCache>
@@ -15342,7 +15378,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B9E993F-B784-7448-B38E-9BEFCF4E7032}">
-  <dimension ref="A1:Q350"/>
+  <dimension ref="A1:Q351"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -30069,6 +30105,49 @@
       <c r="M350" s="19"/>
       <c r="N350" s="19"/>
       <c r="O350">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="351" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A351" s="1">
+        <v>46120</v>
+      </c>
+      <c r="B351" s="2">
+        <v>9</v>
+      </c>
+      <c r="C351">
+        <f t="shared" ref="C351" si="539">SUM(D351:F351)</f>
+        <v>1673</v>
+      </c>
+      <c r="D351">
+        <v>1105</v>
+      </c>
+      <c r="E351">
+        <v>371</v>
+      </c>
+      <c r="F351" s="3">
+        <v>197</v>
+      </c>
+      <c r="G351" s="4">
+        <v>132</v>
+      </c>
+      <c r="H351" s="16">
+        <f t="shared" ref="H351" si="540">SUM(I351:K351)</f>
+        <v>13429</v>
+      </c>
+      <c r="I351" s="5">
+        <v>10445</v>
+      </c>
+      <c r="J351" s="6">
+        <v>1539</v>
+      </c>
+      <c r="K351" s="7">
+        <v>1445</v>
+      </c>
+      <c r="L351" s="19"/>
+      <c r="M351" s="19"/>
+      <c r="N351" s="19"/>
+      <c r="O351">
         <v>31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
line count (lots of new tests)
</commit_message>
<xml_diff>
--- a/Photo Club Hub/Documentation/LineCount.xlsx
+++ b/Photo Club Hub/Documentation/LineCount.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/Photo Club Hub/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B02E41B0-33AA-1D44-9DFE-56683499BF19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDB11D35-FDE3-4944-8AB6-1D1662F316AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="33800" windowHeight="26400" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="33800" windowHeight="26400" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="1" r:id="rId1"/>
@@ -1353,6 +1353,9 @@
                 <c:pt idx="352">
                   <c:v>46141</c:v>
                 </c:pt>
+                <c:pt idx="353">
+                  <c:v>46142</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2420,6 +2423,9 @@
                 </c:pt>
                 <c:pt idx="352" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
                   <c:v>13943</c:v>
+                </c:pt>
+                <c:pt idx="353" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
+                  <c:v>14454</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3526,6 +3532,9 @@
                 <c:pt idx="352">
                   <c:v>46141</c:v>
                 </c:pt>
+                <c:pt idx="353">
+                  <c:v>46142</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4593,6 +4602,9 @@
                 </c:pt>
                 <c:pt idx="352">
                   <c:v>10700</c:v>
+                </c:pt>
+                <c:pt idx="353">
+                  <c:v>11014</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5701,6 +5713,9 @@
                 <c:pt idx="352">
                   <c:v>46141</c:v>
                 </c:pt>
+                <c:pt idx="353">
+                  <c:v>46142</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6768,6 +6783,9 @@
                 </c:pt>
                 <c:pt idx="352">
                   <c:v>1725</c:v>
+                </c:pt>
+                <c:pt idx="353">
+                  <c:v>1838</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7895,6 +7913,9 @@
                 <c:pt idx="352">
                   <c:v>46141</c:v>
                 </c:pt>
+                <c:pt idx="353">
+                  <c:v>46142</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -8962,6 +8983,9 @@
                 </c:pt>
                 <c:pt idx="352">
                   <c:v>1518</c:v>
+                </c:pt>
+                <c:pt idx="353">
+                  <c:v>1602</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10452,6 +10476,9 @@
                 <c:pt idx="352">
                   <c:v>46141</c:v>
                 </c:pt>
+                <c:pt idx="353">
+                  <c:v>46142</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -11518,6 +11545,9 @@
                   <c:v>135</c:v>
                 </c:pt>
                 <c:pt idx="352">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="353">
                   <c:v>135</c:v>
                 </c:pt>
               </c:numCache>
@@ -12628,6 +12658,9 @@
                 <c:pt idx="352">
                   <c:v>46141</c:v>
                 </c:pt>
+                <c:pt idx="353">
+                  <c:v>46142</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -13695,6 +13728,9 @@
                 </c:pt>
                 <c:pt idx="352">
                   <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="353">
+                  <c:v>60</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -15522,7 +15558,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B9E993F-B784-7448-B38E-9BEFCF4E7032}">
-  <dimension ref="A1:Q355"/>
+  <dimension ref="A1:Q356"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -30465,6 +30501,49 @@
       <c r="N355" s="19"/>
       <c r="O355">
         <v>32</v>
+      </c>
+    </row>
+    <row r="356" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A356" s="1">
+        <v>46142</v>
+      </c>
+      <c r="B356" s="2">
+        <v>9</v>
+      </c>
+      <c r="C356">
+        <f t="shared" ref="C356" si="549">SUM(D356:F356)</f>
+        <v>1673</v>
+      </c>
+      <c r="D356">
+        <v>1105</v>
+      </c>
+      <c r="E356">
+        <v>371</v>
+      </c>
+      <c r="F356" s="3">
+        <v>197</v>
+      </c>
+      <c r="G356" s="4">
+        <v>135</v>
+      </c>
+      <c r="H356" s="16">
+        <f t="shared" ref="H356" si="550">SUM(I356:K356)</f>
+        <v>14454</v>
+      </c>
+      <c r="I356" s="5">
+        <v>11014</v>
+      </c>
+      <c r="J356" s="6">
+        <v>1838</v>
+      </c>
+      <c r="K356" s="7">
+        <v>1602</v>
+      </c>
+      <c r="L356" s="19"/>
+      <c r="M356" s="19"/>
+      <c r="N356" s="19"/>
+      <c r="O356">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Line count Fix: #760
</commit_message>
<xml_diff>
--- a/Photo Club Hub/Documentation/LineCount.xlsx
+++ b/Photo Club Hub/Documentation/LineCount.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/Photo Club Hub/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F972506D-2062-5F4D-BFCF-9B10120B90D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AECDEC3B-A698-8F43-B0D3-8244C09DA573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="1" r:id="rId1"/>
@@ -1356,6 +1356,9 @@
                 <c:pt idx="353">
                   <c:v>46144</c:v>
                 </c:pt>
+                <c:pt idx="354">
+                  <c:v>46145</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2425,7 +2428,10 @@
                   <c:v>13943</c:v>
                 </c:pt>
                 <c:pt idx="353" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
-                  <c:v>14776</c:v>
+                  <c:v>14806</c:v>
+                </c:pt>
+                <c:pt idx="354" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
+                  <c:v>15017</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3535,6 +3541,9 @@
                 <c:pt idx="353">
                   <c:v>46144</c:v>
                 </c:pt>
+                <c:pt idx="354">
+                  <c:v>46145</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4605,6 +4614,9 @@
                 </c:pt>
                 <c:pt idx="353">
                   <c:v>11185</c:v>
+                </c:pt>
+                <c:pt idx="354">
+                  <c:v>11318</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5716,6 +5728,9 @@
                 <c:pt idx="353">
                   <c:v>46144</c:v>
                 </c:pt>
+                <c:pt idx="354">
+                  <c:v>46145</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6786,6 +6801,9 @@
                 </c:pt>
                 <c:pt idx="353">
                   <c:v>1971</c:v>
+                </c:pt>
+                <c:pt idx="354">
+                  <c:v>2041</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7916,6 +7934,9 @@
                 <c:pt idx="353">
                   <c:v>46144</c:v>
                 </c:pt>
+                <c:pt idx="354">
+                  <c:v>46145</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -8986,6 +9007,9 @@
                 </c:pt>
                 <c:pt idx="353">
                   <c:v>1650</c:v>
+                </c:pt>
+                <c:pt idx="354">
+                  <c:v>1658</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9078,7 +9102,7 @@
         <c:axId val="1582338719"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="15000"/>
+          <c:max val="15500"/>
           <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -10479,6 +10503,9 @@
                 <c:pt idx="353">
                   <c:v>46144</c:v>
                 </c:pt>
+                <c:pt idx="354">
+                  <c:v>46145</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -11548,6 +11575,9 @@
                   <c:v>135</c:v>
                 </c:pt>
                 <c:pt idx="353">
+                  <c:v>143</c:v>
+                </c:pt>
+                <c:pt idx="354">
                   <c:v>143</c:v>
                 </c:pt>
               </c:numCache>
@@ -12661,6 +12691,9 @@
                 <c:pt idx="353">
                   <c:v>46144</c:v>
                 </c:pt>
+                <c:pt idx="354">
+                  <c:v>46145</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -13730,6 +13763,9 @@
                   <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="353">
+                  <c:v>68</c:v>
+                </c:pt>
+                <c:pt idx="354">
                   <c:v>68</c:v>
                 </c:pt>
               </c:numCache>
@@ -15558,7 +15594,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B9E993F-B784-7448-B38E-9BEFCF4E7032}">
-  <dimension ref="A1:Q356"/>
+  <dimension ref="A1:Q357"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -30441,7 +30477,7 @@
         <v>135</v>
       </c>
       <c r="H354" s="16">
-        <f t="shared" ref="H354" si="546">SUM(I354:K354)</f>
+        <f t="shared" ref="H354:H357" si="546">SUM(I354:K354)</f>
         <v>13557</v>
       </c>
       <c r="I354" s="5">
@@ -30484,7 +30520,7 @@
         <v>135</v>
       </c>
       <c r="H355" s="16">
-        <f t="shared" ref="H355" si="548">SUM(I355:K355)</f>
+        <f t="shared" si="546"/>
         <v>13943</v>
       </c>
       <c r="I355" s="5">
@@ -30511,7 +30547,7 @@
         <v>9</v>
       </c>
       <c r="C356">
-        <f t="shared" ref="C356" si="549">SUM(D356:F356)</f>
+        <f t="shared" ref="C356" si="548">SUM(D356:F356)</f>
         <v>1673</v>
       </c>
       <c r="D356">
@@ -30527,7 +30563,8 @@
         <v>143</v>
       </c>
       <c r="H356" s="16">
-        <v>14776</v>
+        <f t="shared" si="546"/>
+        <v>14806</v>
       </c>
       <c r="I356" s="5">
         <v>11185</v>
@@ -30542,6 +30579,49 @@
       <c r="M356" s="19"/>
       <c r="N356" s="19"/>
       <c r="O356">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="357" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A357" s="1">
+        <v>46145</v>
+      </c>
+      <c r="B357" s="2">
+        <v>9</v>
+      </c>
+      <c r="C357">
+        <f t="shared" ref="C357" si="549">SUM(D357:F357)</f>
+        <v>1673</v>
+      </c>
+      <c r="D357">
+        <v>1105</v>
+      </c>
+      <c r="E357">
+        <v>371</v>
+      </c>
+      <c r="F357" s="3">
+        <v>197</v>
+      </c>
+      <c r="G357" s="4">
+        <v>143</v>
+      </c>
+      <c r="H357" s="16">
+        <f t="shared" si="546"/>
+        <v>15017</v>
+      </c>
+      <c r="I357" s="5">
+        <v>11318</v>
+      </c>
+      <c r="J357" s="6">
+        <v>2041</v>
+      </c>
+      <c r="K357" s="7">
+        <v>1658</v>
+      </c>
+      <c r="L357" s="19"/>
+      <c r="M357" s="19"/>
+      <c r="N357" s="19"/>
+      <c r="O357">
         <v>68</v>
       </c>
     </row>

</xml_diff>

<commit_message>
moved code for ifDebugFatalErrorSpy into another file fixed: #761
</commit_message>
<xml_diff>
--- a/Photo Club Hub/Documentation/LineCount.xlsx
+++ b/Photo Club Hub/Documentation/LineCount.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/Photo Club Hub/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AECDEC3B-A698-8F43-B0D3-8244C09DA573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D8E072-CF90-6A4A-922C-A7157D9DE1BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" activeTab="1" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="19400" windowHeight="16660" xr2:uid="{1D5C550A-6212-F143-B3FD-423F82763F19}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="1" r:id="rId1"/>
@@ -1359,6 +1359,9 @@
                 <c:pt idx="354">
                   <c:v>46145</c:v>
                 </c:pt>
+                <c:pt idx="355">
+                  <c:v>46146</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2432,6 +2435,9 @@
                 </c:pt>
                 <c:pt idx="354" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
                   <c:v>15017</c:v>
+                </c:pt>
+                <c:pt idx="355" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ ">
+                  <c:v>15174</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3544,6 +3550,9 @@
                 <c:pt idx="354">
                   <c:v>46145</c:v>
                 </c:pt>
+                <c:pt idx="355">
+                  <c:v>46146</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4617,6 +4626,9 @@
                 </c:pt>
                 <c:pt idx="354">
                   <c:v>11318</c:v>
+                </c:pt>
+                <c:pt idx="355">
+                  <c:v>11404</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5731,6 +5743,9 @@
                 <c:pt idx="354">
                   <c:v>46145</c:v>
                 </c:pt>
+                <c:pt idx="355">
+                  <c:v>46146</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -6804,6 +6819,9 @@
                 </c:pt>
                 <c:pt idx="354">
                   <c:v>2041</c:v>
+                </c:pt>
+                <c:pt idx="355">
+                  <c:v>2082</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7937,6 +7955,9 @@
                 <c:pt idx="354">
                   <c:v>46145</c:v>
                 </c:pt>
+                <c:pt idx="355">
+                  <c:v>46146</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -9010,6 +9031,9 @@
                 </c:pt>
                 <c:pt idx="354">
                   <c:v>1658</c:v>
+                </c:pt>
+                <c:pt idx="355">
+                  <c:v>1688</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10506,6 +10530,9 @@
                 <c:pt idx="354">
                   <c:v>46145</c:v>
                 </c:pt>
+                <c:pt idx="355">
+                  <c:v>46146</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -11579,6 +11606,9 @@
                 </c:pt>
                 <c:pt idx="354">
                   <c:v>143</c:v>
+                </c:pt>
+                <c:pt idx="355">
+                  <c:v>144</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12694,6 +12724,9 @@
                 <c:pt idx="354">
                   <c:v>46145</c:v>
                 </c:pt>
+                <c:pt idx="355">
+                  <c:v>46146</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -13767,6 +13800,9 @@
                 </c:pt>
                 <c:pt idx="354">
                   <c:v>68</c:v>
+                </c:pt>
+                <c:pt idx="355">
+                  <c:v>69</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -15594,7 +15630,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B9E993F-B784-7448-B38E-9BEFCF4E7032}">
-  <dimension ref="A1:Q357"/>
+  <dimension ref="A1:Q358"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -30623,6 +30659,49 @@
       <c r="N357" s="19"/>
       <c r="O357">
         <v>68</v>
+      </c>
+    </row>
+    <row r="358" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A358" s="1">
+        <v>46146</v>
+      </c>
+      <c r="B358" s="2">
+        <v>9</v>
+      </c>
+      <c r="C358">
+        <f t="shared" ref="C358" si="550">SUM(D358:F358)</f>
+        <v>1673</v>
+      </c>
+      <c r="D358">
+        <v>1105</v>
+      </c>
+      <c r="E358">
+        <v>371</v>
+      </c>
+      <c r="F358" s="3">
+        <v>197</v>
+      </c>
+      <c r="G358" s="4">
+        <v>144</v>
+      </c>
+      <c r="H358" s="16">
+        <f t="shared" ref="H358" si="551">SUM(I358:K358)</f>
+        <v>15174</v>
+      </c>
+      <c r="I358" s="5">
+        <v>11404</v>
+      </c>
+      <c r="J358" s="6">
+        <v>2082</v>
+      </c>
+      <c r="K358" s="7">
+        <v>1688</v>
+      </c>
+      <c r="L358" s="19"/>
+      <c r="M358" s="19"/>
+      <c r="N358" s="19"/>
+      <c r="O358">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>